<commit_message>
Fix name: Jenny Louis -> Jenny Lui in RACI map
</commit_message>
<xml_diff>
--- a/marketing-ownership-map.xlsx
+++ b/marketing-ownership-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LRUSIN~1\AppData\Local\Temp\claude\c--Users-lrusinova-OneDrive---QuickBase-Documents-Project-Management-MCP\abf0f386-0ae7-411b-800d-e81e7586b212\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B66F7592-3596-4883-B9B8-8254B28DD6DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA43AA72-5732-48C6-ABC7-8FB3A181BA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{840B5537-3834-4E38-8A1A-8FEB33A66693}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{ADBF567C-1F4C-4A6D-87E4-148EBC33D2C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Ownership Matrix" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
     <author>Rusinova, Luiza</author>
   </authors>
   <commentList>
-    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{537CC844-9E50-46D8-9FF4-CC6B05AFF905}">
+    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{7DE34742-5DEC-4463-8B60-85207869E3E0}">
       <text>
         <r>
           <rPr>
@@ -59,7 +59,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{6F212F61-0CA5-408D-B0FA-B3DFE2F37743}">
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{1F55DDC0-4776-414A-A47D-5D622508EEEC}">
       <text>
         <r>
           <rPr>
@@ -73,7 +73,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{82D430CA-3774-44D6-90F6-08E87B2078DC}">
+    <comment ref="E6" authorId="0" shapeId="0" xr:uid="{A17C0921-6D73-4F93-A751-6AAF90B505F6}">
       <text>
         <r>
           <rPr>
@@ -88,7 +88,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{331E90AF-3F7F-4F30-9B12-9651A48A50A6}">
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{1A2D261A-EBA8-438C-8232-F51E06F29A66}">
       <text>
         <r>
           <rPr>
@@ -102,7 +102,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G6" authorId="0" shapeId="0" xr:uid="{E89D89C4-CBEF-4E89-A579-717992B71D85}">
+    <comment ref="G6" authorId="0" shapeId="0" xr:uid="{3758F9D8-E94E-4AE7-86AE-885C3DC16F1B}">
       <text>
         <r>
           <rPr>
@@ -117,7 +117,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H6" authorId="0" shapeId="0" xr:uid="{B176D216-DA64-419E-B317-56E04C1731BA}">
+    <comment ref="H6" authorId="0" shapeId="0" xr:uid="{9889D2A3-424B-498F-B837-B1FF5785345D}">
       <text>
         <r>
           <rPr>
@@ -131,7 +131,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I6" authorId="0" shapeId="0" xr:uid="{9690C19F-DC72-488B-B312-0CE82DE04F91}">
+    <comment ref="I6" authorId="0" shapeId="0" xr:uid="{38401944-6320-46B0-A577-662AEB74C926}">
       <text>
         <r>
           <rPr>
@@ -145,7 +145,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{99AF020B-A93B-4045-B5A2-96148BB6DAC8}">
+    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{11F5E611-549F-4380-BD99-05759C49E531}">
       <text>
         <r>
           <rPr>
@@ -159,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C7" authorId="0" shapeId="0" xr:uid="{244C2EEC-A1F4-48C8-99A3-875101732B02}">
+    <comment ref="C7" authorId="0" shapeId="0" xr:uid="{85E94519-B74F-4BAD-9CCC-686FAC71D5E5}">
       <text>
         <r>
           <rPr>
@@ -173,7 +173,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{C0E7F949-4263-4A32-9214-1C95163C2014}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{317B8EA8-E95C-446F-A385-C91E9BD8DC0A}">
       <text>
         <r>
           <rPr>
@@ -188,7 +188,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{AB3F0F02-5BF1-401A-8FB8-A0BC41A63489}">
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{40398932-E92F-4AD3-BF07-B7F8483B47A2}">
       <text>
         <r>
           <rPr>
@@ -202,7 +202,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{0149602F-6E3C-4D8D-A3EF-E63F2BE5E422}">
+    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{0164D3B8-C066-4343-886C-A4FBAAE01567}">
       <text>
         <r>
           <rPr>
@@ -216,7 +216,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J7" authorId="0" shapeId="0" xr:uid="{E5A73CA3-DCC7-4F3D-852C-FDC3868330C1}">
+    <comment ref="J7" authorId="0" shapeId="0" xr:uid="{2C4A446B-9C95-4066-A05A-A653C3E5117E}">
       <text>
         <r>
           <rPr>
@@ -230,21 +230,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="C8" authorId="0" shapeId="0" xr:uid="{F7127242-7E7C-4130-AFD0-D5F86FD8FF8E}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Joins the pre-kickoff strategy call (per Jenny Louis, Director of Brand &amp; Creative) to weigh in on positioning before deliverables are scoped.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{3EB93470-340A-47E9-AD0D-FCAC2F41142A}">
+    <comment ref="C8" authorId="0" shapeId="0" xr:uid="{43CB05E5-599B-4245-9EBE-3FCE78B2C63A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Joins the pre-kickoff strategy call (per Jenny Lui, Director of Brand &amp; Creative) to weigh in on positioning before deliverables are scoped.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{7166393F-9E9F-47A3-B599-7ED99CAC399F}">
       <text>
         <r>
           <rPr>
@@ -258,7 +258,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E8" authorId="0" shapeId="0" xr:uid="{CE84555B-30AB-48DF-A6CF-00EA38AB0549}">
+    <comment ref="E8" authorId="0" shapeId="0" xr:uid="{DE347DE8-8893-4B4C-9F30-D50F999594AA}">
       <text>
         <r>
           <rPr>
@@ -272,7 +272,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F8" authorId="0" shapeId="0" xr:uid="{21D46017-1BEA-4A11-8AA7-2738F6765058}">
+    <comment ref="F8" authorId="0" shapeId="0" xr:uid="{13319A90-455A-4F49-B5CF-A96F866D93F8}">
       <text>
         <r>
           <rPr>
@@ -286,7 +286,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G8" authorId="0" shapeId="0" xr:uid="{84964482-1CBE-449E-AF32-80250D4E07AD}">
+    <comment ref="G8" authorId="0" shapeId="0" xr:uid="{5B2EC2F8-1356-478A-B068-56FD7855840C}">
       <text>
         <r>
           <rPr>
@@ -301,7 +301,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H8" authorId="0" shapeId="0" xr:uid="{008E22CB-94FE-4C4D-A874-7C07EBCD9AA0}">
+    <comment ref="H8" authorId="0" shapeId="0" xr:uid="{999108B7-4DCB-40D9-A3B5-840139F8924C}">
       <text>
         <r>
           <rPr>
@@ -315,7 +315,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E9" authorId="0" shapeId="0" xr:uid="{B0703DB3-E497-4F73-9B0C-77CF973B15CD}">
+    <comment ref="E9" authorId="0" shapeId="0" xr:uid="{33F75203-D8BE-4B40-BC0C-32B9DD0123DC}">
       <text>
         <r>
           <rPr>
@@ -329,7 +329,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I9" authorId="0" shapeId="0" xr:uid="{1D75D182-DA89-47F5-8CF1-762D86E9F9F1}">
+    <comment ref="I9" authorId="0" shapeId="0" xr:uid="{8110718A-FD8C-4F26-962A-FB3B981A72A9}">
       <text>
         <r>
           <rPr>
@@ -343,7 +343,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J9" authorId="0" shapeId="0" xr:uid="{0B8F9D5C-C28A-4E81-9381-97D26D7CBAC0}">
+    <comment ref="J9" authorId="0" shapeId="0" xr:uid="{95B0933E-BBB8-4D96-8076-098036954215}">
       <text>
         <r>
           <rPr>
@@ -357,7 +357,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C11" authorId="0" shapeId="0" xr:uid="{64264F1A-725F-40EE-B1C8-C8E6B7EA42FF}">
+    <comment ref="C11" authorId="0" shapeId="0" xr:uid="{EADC331C-416C-4F17-9B9C-BA34CDDFBCBD}">
       <text>
         <r>
           <rPr>
@@ -371,7 +371,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F11" authorId="0" shapeId="0" xr:uid="{1C7814D0-32F1-47D5-9A77-7EA9AAEE056D}">
+    <comment ref="F11" authorId="0" shapeId="0" xr:uid="{8E55F199-3381-439E-A1A3-A454146A0859}">
       <text>
         <r>
           <rPr>
@@ -385,7 +385,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G11" authorId="0" shapeId="0" xr:uid="{247902C4-5B4C-4574-89B7-3650BC2F171F}">
+    <comment ref="G11" authorId="0" shapeId="0" xr:uid="{D9989B45-4139-449F-820A-9ECD262FD437}">
       <text>
         <r>
           <rPr>
@@ -400,7 +400,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H11" authorId="0" shapeId="0" xr:uid="{044DB200-6145-48E2-8F2B-5EC4AB9375F8}">
+    <comment ref="H11" authorId="0" shapeId="0" xr:uid="{99762019-B8B0-43BA-AD02-477CA4AAD5A7}">
       <text>
         <r>
           <rPr>
@@ -414,21 +414,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{E4632C3C-DD0D-4C49-8389-3C5B6C3C0663}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Joins the pre-kickoff strategy call (per Jenny Louis, Director of Brand &amp; Creative) to flag creative/asset approach before deliverables are scoped.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G12" authorId="0" shapeId="0" xr:uid="{F65B690C-4B2F-47FD-923F-83C1A39A3283}">
+    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{9DF2B69C-6BF4-4509-B8E3-3AA88B4F5737}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Joins the pre-kickoff strategy call (per Jenny Lui, Director of Brand &amp; Creative) to flag creative/asset approach before deliverables are scoped.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="0" shapeId="0" xr:uid="{F8168D89-53B4-42D3-963F-78054D64C69C}">
       <text>
         <r>
           <rPr>
@@ -442,7 +442,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H12" authorId="0" shapeId="0" xr:uid="{D652496D-D9FD-4804-864C-342320ECC95D}">
+    <comment ref="H12" authorId="0" shapeId="0" xr:uid="{515B47C5-1264-44C3-AA6D-C15829525771}">
       <text>
         <r>
           <rPr>
@@ -456,7 +456,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{7B7E1958-0AC8-414F-9013-744F6B31E672}">
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{DFE3D0E9-B88A-4605-92C2-37F667297B04}">
       <text>
         <r>
           <rPr>
@@ -470,7 +470,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E13" authorId="0" shapeId="0" xr:uid="{D0D14E1E-F28F-4F30-B7E8-4481051AE8CE}">
+    <comment ref="E13" authorId="0" shapeId="0" xr:uid="{ED87AD16-284E-4850-8D5D-949A48C6C6D5}">
       <text>
         <r>
           <rPr>
@@ -484,7 +484,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F13" authorId="0" shapeId="0" xr:uid="{02558303-BFC1-4338-841E-6554164BA0D1}">
+    <comment ref="F13" authorId="0" shapeId="0" xr:uid="{469F0668-0830-4B7C-9281-30F265F7934C}">
       <text>
         <r>
           <rPr>
@@ -498,7 +498,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G13" authorId="0" shapeId="0" xr:uid="{69E31930-E18F-4B94-90AF-3D8D8FB2A33B}">
+    <comment ref="G13" authorId="0" shapeId="0" xr:uid="{741E7FFE-A857-4230-BD12-64AC5A853284}">
       <text>
         <r>
           <rPr>
@@ -512,7 +512,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H13" authorId="0" shapeId="0" xr:uid="{745FA499-7B64-40B2-AFE2-E2B9B444A59E}">
+    <comment ref="H13" authorId="0" shapeId="0" xr:uid="{506A5A7F-1B18-4F39-B012-2FECC80679F8}">
       <text>
         <r>
           <rPr>
@@ -526,7 +526,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J13" authorId="0" shapeId="0" xr:uid="{CF5A20AA-A4D0-42A2-B968-C704C4FF399B}">
+    <comment ref="J13" authorId="0" shapeId="0" xr:uid="{F60BB9C5-FEBB-4D7B-AAEF-FB3E28C8CF30}">
       <text>
         <r>
           <rPr>
@@ -540,7 +540,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E14" authorId="0" shapeId="0" xr:uid="{78AE6D5A-B632-4758-9715-8CCB2F4545BE}">
+    <comment ref="E14" authorId="0" shapeId="0" xr:uid="{71AF8E85-4AC1-4041-B5BD-D4AF2909CB10}">
       <text>
         <r>
           <rPr>
@@ -554,7 +554,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G14" authorId="0" shapeId="0" xr:uid="{32B96530-C76B-4F33-A4C8-97006B46F8C4}">
+    <comment ref="G14" authorId="0" shapeId="0" xr:uid="{39BBF026-D7E0-4BFE-9AF3-13F4FBAD97B7}">
       <text>
         <r>
           <rPr>
@@ -568,7 +568,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H14" authorId="0" shapeId="0" xr:uid="{2F270CF0-A03A-4965-8E41-2AB8FE7CB995}">
+    <comment ref="H14" authorId="0" shapeId="0" xr:uid="{16951E65-2C5C-4D7E-B44A-8E5481B7CE66}">
       <text>
         <r>
           <rPr>
@@ -582,7 +582,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I14" authorId="0" shapeId="0" xr:uid="{C2A08AE6-E0A3-443F-93AE-CDC84C4995CA}">
+    <comment ref="I14" authorId="0" shapeId="0" xr:uid="{71724FF0-A5FB-4610-A97D-C1F31AC656B9}">
       <text>
         <r>
           <rPr>
@@ -596,7 +596,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J14" authorId="0" shapeId="0" xr:uid="{4CB40028-B8FE-4558-98EE-3E69DBCCC631}">
+    <comment ref="J14" authorId="0" shapeId="0" xr:uid="{EC2A2EAE-9C6F-4027-B167-9F5EF9CD131C}">
       <text>
         <r>
           <rPr>
@@ -610,7 +610,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E16" authorId="0" shapeId="0" xr:uid="{96A94C7D-46EC-4BF2-8F2C-74ED96260B02}">
+    <comment ref="E16" authorId="0" shapeId="0" xr:uid="{F7EA35BF-567D-49FB-A636-5609FDBA4BF7}">
       <text>
         <r>
           <rPr>
@@ -624,7 +624,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G16" authorId="0" shapeId="0" xr:uid="{16254745-3B74-4D44-8AB3-6FD6BBDCE3B5}">
+    <comment ref="G16" authorId="0" shapeId="0" xr:uid="{E1C0B952-D615-4D28-AC53-2239E64B266D}">
       <text>
         <r>
           <rPr>
@@ -638,7 +638,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I16" authorId="0" shapeId="0" xr:uid="{46B7FE16-165B-426E-8998-55B1E16A5959}">
+    <comment ref="I16" authorId="0" shapeId="0" xr:uid="{A1CF2403-1105-4A6F-ADFE-6B6F8EBD6E8F}">
       <text>
         <r>
           <rPr>
@@ -652,7 +652,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J16" authorId="0" shapeId="0" xr:uid="{7C409EAF-234B-4921-A64D-FEA7C4BDFAF7}">
+    <comment ref="J16" authorId="0" shapeId="0" xr:uid="{01B3E2F4-70CA-4151-8C8F-F874997D91B8}">
       <text>
         <r>
           <rPr>
@@ -666,7 +666,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E17" authorId="0" shapeId="0" xr:uid="{B6129FD6-7E70-44D0-B703-1D8BA2DAD6A5}">
+    <comment ref="E17" authorId="0" shapeId="0" xr:uid="{CB4F56AF-9363-4631-A8CC-0F36B848F7F9}">
       <text>
         <r>
           <rPr>
@@ -680,7 +680,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G17" authorId="0" shapeId="0" xr:uid="{73570073-FB44-4785-9E15-C238AFD19454}">
+    <comment ref="G17" authorId="0" shapeId="0" xr:uid="{21EC90F2-E20F-490E-924D-0DE554DBA751}">
       <text>
         <r>
           <rPr>
@@ -694,7 +694,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I17" authorId="0" shapeId="0" xr:uid="{A0565A38-78F0-4AFF-8A04-45F01D315FB6}">
+    <comment ref="I17" authorId="0" shapeId="0" xr:uid="{B0C8AF5A-A765-43F4-92C9-1171DDC9C0FE}">
       <text>
         <r>
           <rPr>
@@ -708,7 +708,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J17" authorId="0" shapeId="0" xr:uid="{28330EC4-62B5-4198-A0C5-4E764F74ED65}">
+    <comment ref="J17" authorId="0" shapeId="0" xr:uid="{44891C13-D6E9-4CD1-83BF-52E9DE82BBFA}">
       <text>
         <r>
           <rPr>
@@ -722,7 +722,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{39CB1A88-85BE-4DB6-94C5-2B2089DE28D9}">
+    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{2A6B3B22-F263-4E2F-845C-6FAC90DE278C}">
       <text>
         <r>
           <rPr>
@@ -736,7 +736,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E18" authorId="0" shapeId="0" xr:uid="{5FBBD009-1C3B-4654-97A0-CC9D7EE3CEE1}">
+    <comment ref="E18" authorId="0" shapeId="0" xr:uid="{87576241-A281-419B-8CA3-4AD2806EB415}">
       <text>
         <r>
           <rPr>
@@ -750,7 +750,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G18" authorId="0" shapeId="0" xr:uid="{D051E8E3-2846-4589-8F9E-CFE4380E61E1}">
+    <comment ref="G18" authorId="0" shapeId="0" xr:uid="{8E972169-81C7-4529-8EEB-B09EFDA72875}">
       <text>
         <r>
           <rPr>
@@ -764,7 +764,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H18" authorId="0" shapeId="0" xr:uid="{42AE314B-8207-49F3-A1A3-313B0CBAE351}">
+    <comment ref="H18" authorId="0" shapeId="0" xr:uid="{686ACD90-4B53-4D53-85B8-5BDF1EE87A1D}">
       <text>
         <r>
           <rPr>
@@ -778,7 +778,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I18" authorId="0" shapeId="0" xr:uid="{99BD5D43-E37F-47CA-833E-F63213850D81}">
+    <comment ref="I18" authorId="0" shapeId="0" xr:uid="{F9439D3B-B7DF-448E-B36C-2BA287AD8F4E}">
       <text>
         <r>
           <rPr>
@@ -792,7 +792,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J18" authorId="0" shapeId="0" xr:uid="{0BCCF6FD-1D9D-4F15-BCD2-0DE513F17FA0}">
+    <comment ref="J18" authorId="0" shapeId="0" xr:uid="{2A5EA72C-09E9-4636-9174-F5102C14789A}">
       <text>
         <r>
           <rPr>
@@ -806,7 +806,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E19" authorId="0" shapeId="0" xr:uid="{8F5A6F63-F3BB-4F0F-8F41-09295BD3FBF5}">
+    <comment ref="E19" authorId="0" shapeId="0" xr:uid="{3E07ED08-D6D5-4BE1-A5FB-45E52B54EF3C}">
       <text>
         <r>
           <rPr>
@@ -820,7 +820,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G19" authorId="0" shapeId="0" xr:uid="{C085B643-144C-45A2-9A79-5159E7E0EF6E}">
+    <comment ref="G19" authorId="0" shapeId="0" xr:uid="{02F9447F-CF33-4050-9CAF-C832B8E2B20E}">
       <text>
         <r>
           <rPr>
@@ -834,7 +834,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I19" authorId="0" shapeId="0" xr:uid="{159395E5-59E0-45CD-908F-D672660178F4}">
+    <comment ref="I19" authorId="0" shapeId="0" xr:uid="{B798E47C-E88D-4FBC-9C59-AEC09262D02E}">
       <text>
         <r>
           <rPr>
@@ -848,7 +848,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J19" authorId="0" shapeId="0" xr:uid="{D3FA42B5-9709-4AA7-AB7D-E20D8FBECFD9}">
+    <comment ref="J19" authorId="0" shapeId="0" xr:uid="{F25D2C4E-ECFA-4243-B17E-A03791258CC9}">
       <text>
         <r>
           <rPr>
@@ -862,7 +862,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{E2A77803-2CCA-4C42-BDE9-A1D792EC649D}">
+    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{0ADAE55F-8485-416C-A564-C5990FFCCC24}">
       <text>
         <r>
           <rPr>
@@ -877,7 +877,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G20" authorId="0" shapeId="0" xr:uid="{E1FDDC36-F902-47D7-8525-B9BDF666DA77}">
+    <comment ref="G20" authorId="0" shapeId="0" xr:uid="{23ACAD03-0F8C-47F8-97F1-69B908AE1E3C}">
       <text>
         <r>
           <rPr>
@@ -891,7 +891,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H20" authorId="0" shapeId="0" xr:uid="{20A8D9BA-7FDA-4B5D-AA36-8BCD988D9862}">
+    <comment ref="H20" authorId="0" shapeId="0" xr:uid="{38F4B2A0-45DC-4C3E-B16B-B241CEA0FD9A}">
       <text>
         <r>
           <rPr>
@@ -905,7 +905,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I20" authorId="0" shapeId="0" xr:uid="{EEAEA712-3626-4BC7-9F87-A062314BB8B1}">
+    <comment ref="I20" authorId="0" shapeId="0" xr:uid="{E9A55A74-131D-4F52-A5B5-4FDA6CE86108}">
       <text>
         <r>
           <rPr>
@@ -919,7 +919,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J20" authorId="0" shapeId="0" xr:uid="{63C85853-5B48-4395-AB24-28B65E8173B3}">
+    <comment ref="J20" authorId="0" shapeId="0" xr:uid="{BC067597-70EE-4BB8-A26B-5E5FC3BAAEB1}">
       <text>
         <r>
           <rPr>
@@ -933,7 +933,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{AF6DDDBB-AECF-4960-86FE-262663ED9873}">
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{F08F3952-3542-4117-8485-830BE8FCA06D}">
       <text>
         <r>
           <rPr>
@@ -947,7 +947,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{4CF74813-4053-4945-9EF8-B2D3A9A2491D}">
+    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{7C462FFB-73AE-4BE5-9FD1-EC67474F0DC5}">
       <text>
         <r>
           <rPr>
@@ -961,7 +961,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G21" authorId="0" shapeId="0" xr:uid="{E44A1D20-365F-4120-ACFE-7176579BC94F}">
+    <comment ref="G21" authorId="0" shapeId="0" xr:uid="{4A42E715-7CCB-44EA-954D-26109F86362C}">
       <text>
         <r>
           <rPr>
@@ -975,7 +975,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H21" authorId="0" shapeId="0" xr:uid="{632F8174-ADC9-4703-BAE4-43566DCA2C1C}">
+    <comment ref="H21" authorId="0" shapeId="0" xr:uid="{DCEFA3CA-FB85-4216-B472-73AB3ED5F79E}">
       <text>
         <r>
           <rPr>
@@ -989,7 +989,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I21" authorId="0" shapeId="0" xr:uid="{4A864DCF-3D64-43F5-A4A9-AA9F933F697C}">
+    <comment ref="I21" authorId="0" shapeId="0" xr:uid="{CE500F7A-CD50-457F-A93A-02798409260F}">
       <text>
         <r>
           <rPr>
@@ -1003,7 +1003,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J21" authorId="0" shapeId="0" xr:uid="{0213CCD2-6278-4D4A-A112-1BEB1C13F6EA}">
+    <comment ref="J21" authorId="0" shapeId="0" xr:uid="{51C3405B-7E23-4112-9180-B180A6054D9F}">
       <text>
         <r>
           <rPr>
@@ -1017,7 +1017,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{9B4E76DB-493B-453C-BE1D-A7513C517121}">
+    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{C9B9B515-A8D1-403C-BC99-4E59D4C526ED}">
       <text>
         <r>
           <rPr>
@@ -1031,7 +1031,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G22" authorId="0" shapeId="0" xr:uid="{0AE9675D-176A-45A1-9436-F9F80163F466}">
+    <comment ref="G22" authorId="0" shapeId="0" xr:uid="{7C570F8B-0E99-4C9F-A396-BABE9CCFBD5D}">
       <text>
         <r>
           <rPr>
@@ -1045,7 +1045,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H22" authorId="0" shapeId="0" xr:uid="{781EA18D-A7C1-43A8-B316-C04D41FF310B}">
+    <comment ref="H22" authorId="0" shapeId="0" xr:uid="{F228CBF0-7968-4EFD-A862-F297242FF5D7}">
       <text>
         <r>
           <rPr>
@@ -1059,7 +1059,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I22" authorId="0" shapeId="0" xr:uid="{CAACBFB2-E520-4EB9-B76B-D55F493177C5}">
+    <comment ref="I22" authorId="0" shapeId="0" xr:uid="{460B977E-59AE-4C96-BD7F-8C80D0B84E89}">
       <text>
         <r>
           <rPr>
@@ -1073,7 +1073,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J22" authorId="0" shapeId="0" xr:uid="{CA260731-A31E-4733-8EA4-FB6069D0EE20}">
+    <comment ref="J22" authorId="0" shapeId="0" xr:uid="{A6F490CA-7473-4315-9BB0-C2D33732A957}">
       <text>
         <r>
           <rPr>
@@ -1087,7 +1087,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{66027402-F58C-4267-A7A5-F4BC145C98A6}">
+    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{BA06F242-7739-4810-BE9B-5B53F952B6DC}">
       <text>
         <r>
           <rPr>
@@ -1101,7 +1101,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{A6C2E588-4AD8-48A7-A44E-DCBB1CF961AB}">
+    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{9C616769-CB89-4ABE-8833-49A09CC8AFE4}">
       <text>
         <r>
           <rPr>
@@ -1116,7 +1116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G23" authorId="0" shapeId="0" xr:uid="{61C975E0-12F2-4D3B-8CC7-A8441CACB557}">
+    <comment ref="G23" authorId="0" shapeId="0" xr:uid="{67D2B3D2-A257-4999-BF6A-73ADCC706A36}">
       <text>
         <r>
           <rPr>
@@ -1130,7 +1130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H23" authorId="0" shapeId="0" xr:uid="{FCBC009D-0370-432E-A966-5BB1A5FA4791}">
+    <comment ref="H23" authorId="0" shapeId="0" xr:uid="{ED320130-4A68-4633-A508-DB772BBB91B6}">
       <text>
         <r>
           <rPr>
@@ -1144,7 +1144,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I23" authorId="0" shapeId="0" xr:uid="{D08FB474-17BF-47E7-9395-5B36ECB3AF0D}">
+    <comment ref="I23" authorId="0" shapeId="0" xr:uid="{AED8018E-1FC0-4A94-AEDB-1CBFBA4EBA0B}">
       <text>
         <r>
           <rPr>
@@ -1158,7 +1158,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J23" authorId="0" shapeId="0" xr:uid="{153A8F0B-DD7D-4B6E-A124-CACDA936DC1B}">
+    <comment ref="J23" authorId="0" shapeId="0" xr:uid="{41A37461-2D61-452D-8041-573620C05AEB}">
       <text>
         <r>
           <rPr>
@@ -1173,7 +1173,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C25" authorId="0" shapeId="0" xr:uid="{DCEA9FC0-A711-4A28-BE24-E33F95C9A4AE}">
+    <comment ref="C25" authorId="0" shapeId="0" xr:uid="{92E9143E-8F37-4D34-9CF3-86BC1DA90459}">
       <text>
         <r>
           <rPr>
@@ -1187,7 +1187,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E25" authorId="0" shapeId="0" xr:uid="{4873C3D9-F2B2-4B2E-9464-9A0F2AA75777}">
+    <comment ref="E25" authorId="0" shapeId="0" xr:uid="{228EC8C7-FDAE-41E6-9109-8CA94006FF6E}">
       <text>
         <r>
           <rPr>
@@ -1201,7 +1201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F25" authorId="0" shapeId="0" xr:uid="{182926B4-4A8F-4282-8471-D979DD21E028}">
+    <comment ref="F25" authorId="0" shapeId="0" xr:uid="{FD18C5BF-CDBA-4A3F-9116-32A11663FD00}">
       <text>
         <r>
           <rPr>
@@ -1215,7 +1215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G25" authorId="0" shapeId="0" xr:uid="{9E2B77B5-F838-4460-AF4B-F7B915421F54}">
+    <comment ref="G25" authorId="0" shapeId="0" xr:uid="{B3B912FB-C979-44DE-BBF0-100A50BDA736}">
       <text>
         <r>
           <rPr>
@@ -1229,7 +1229,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I25" authorId="0" shapeId="0" xr:uid="{68F72275-02B1-43FF-9F0D-95D59EC8A714}">
+    <comment ref="I25" authorId="0" shapeId="0" xr:uid="{BBD7E4AF-8E9B-42A5-B5E8-7A66CD2840B1}">
       <text>
         <r>
           <rPr>
@@ -1243,7 +1243,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{196F64AB-7159-4E64-A576-3F1E19EC3BBD}">
+    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{3E38B2B0-0B6F-41AB-97F9-E3F267B3AB8B}">
       <text>
         <r>
           <rPr>
@@ -1477,7 +1477,7 @@
     <t>Reports channel performance against targets.</t>
   </si>
   <si>
-    <t>Joins the pre-kickoff strategy call (per Jenny Louis, Director of Brand &amp; Creative) to weigh in on positioning before deliverables are scoped.</t>
+    <t>Joins the pre-kickoff strategy call (per Jenny Lui, Director of Brand &amp; Creative) to weigh in on positioning before deliverables are scoped.</t>
   </si>
   <si>
     <t>Owns narrative, positioning, and messaging architecture.</t>
@@ -1522,7 +1522,7 @@
     <t>Incorporates review feedback.</t>
   </si>
   <si>
-    <t>Joins the pre-kickoff strategy call (per Jenny Louis, Director of Brand &amp; Creative) to flag creative/asset approach before deliverables are scoped.</t>
+    <t>Joins the pre-kickoff strategy call (per Jenny Lui, Director of Brand &amp; Creative) to flag creative/asset approach before deliverables are scoped.</t>
   </si>
   <si>
     <t>Produces visual/design assets.</t>
@@ -1916,16 +1916,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C61C7A6C-7615-431F-B40C-EDA7291A25D3}" name="OwnershipData" displayName="OwnershipData" ref="A1:G137" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:G137" xr:uid="{C61C7A6C-7615-431F-B40C-EDA7291A25D3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8C8C3D2D-8A01-48A6-BE8E-E2D22875FC43}" name="OwnershipData" displayName="OwnershipData" ref="A1:G137" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:G137" xr:uid="{8C8C3D2D-8A01-48A6-BE8E-E2D22875FC43}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{9C50D4B1-563D-49A8-A88E-CDDF693E3B01}" name="Team"/>
-    <tableColumn id="2" xr3:uid="{8AA70762-6D6D-44A2-AD93-6E4537C4880A}" name="Team Group"/>
-    <tableColumn id="3" xr3:uid="{BD8E6D9B-D254-4795-A30D-637C62BC3A3C}" name="Stage"/>
-    <tableColumn id="4" xr3:uid="{5F14F368-29C6-4407-8F4F-7C407AABB0D3}" name="RACI"/>
-    <tableColumn id="5" xr3:uid="{E0C6DE87-E8CB-467E-AD12-9038663D1CC8}" name="Note"/>
-    <tableColumn id="6" xr3:uid="{41640DA7-CA11-4CF9-A788-DDCE1BFD765F}" name="Conflict"/>
-    <tableColumn id="7" xr3:uid="{E5231930-1FAF-43DC-8BD2-D868EE2FBF1C}" name="Conflict Note"/>
+    <tableColumn id="1" xr3:uid="{2E2C7524-55A1-4FC6-8475-026F4FF2919B}" name="Team"/>
+    <tableColumn id="2" xr3:uid="{95AA5A62-A822-47CE-94BC-92103EFA0850}" name="Team Group"/>
+    <tableColumn id="3" xr3:uid="{8E405F79-F8FD-482B-9EAB-EAD9BB0CC229}" name="Stage"/>
+    <tableColumn id="4" xr3:uid="{DF47C2C1-74BF-4907-B0CD-D8730D8A44AB}" name="RACI"/>
+    <tableColumn id="5" xr3:uid="{2FA533DE-65FC-4A8B-85F8-91E049006FFE}" name="Note"/>
+    <tableColumn id="6" xr3:uid="{A38E4250-D730-45A0-80E7-5CF20C7791C7}" name="Conflict"/>
+    <tableColumn id="7" xr3:uid="{11D74464-C59C-44BC-8DBB-C0A0B1B97466}" name="Conflict Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2247,7 +2247,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{907F1F04-6417-4FE3-8644-27B0B8304B53}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01CE1FA-930D-4760-AC02-5FF3A6A920DD}">
   <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2877,7 +2877,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A676F9BA-A5F2-43F6-86CD-E44727B2CB39}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95E7F510-9BA2-404C-9032-21C8FA09436C}">
   <dimension ref="A1:G137"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>

</xml_diff>

<commit_message>
Add Project Type Guide tab: stage applicability (Full/Light/Skip) by project type
</commit_message>
<xml_diff>
--- a/marketing-ownership-map.xlsx
+++ b/marketing-ownership-map.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LRUSIN~1\AppData\Local\Temp\claude\c--Users-lrusinova-OneDrive---QuickBase-Documents-Project-Management-MCP\abf0f386-0ae7-411b-800d-e81e7586b212\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804F8EB9-DE6B-45CF-9EC8-13B68BADB024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA708C2-042D-4FF9-B4C2-97C5AB71F5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{6BE01299-3AA2-44C9-B560-36F384A9188D}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{6BE01299-3AA2-44C9-B560-36F384A9188D}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary" sheetId="3" r:id="rId1"/>
-    <sheet name="Ownership Matrix" sheetId="1" r:id="rId2"/>
-    <sheet name="Data" sheetId="2" r:id="rId3"/>
+    <sheet name="Project Type Guide" sheetId="4" r:id="rId2"/>
+    <sheet name="Ownership Matrix" sheetId="1" r:id="rId3"/>
+    <sheet name="Data" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1263,7 +1264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="210">
   <si>
     <t>Marketing Ownership Map - RACI Matrix (Working Draft)</t>
   </si>
@@ -1788,13 +1789,118 @@
   </si>
   <si>
     <t>Active Teams</t>
+  </si>
+  <si>
+    <t>Project Type Guide - How Much of the Process Applies</t>
+  </si>
+  <si>
+    <t>The Ownership Matrix's 8 stages are built around a full Launch. Most other project types only need some of them - this shows how much of each stage actually applies, so you're not running the full process for a one-off creative request or a blog post.</t>
+  </si>
+  <si>
+    <t>Project Type</t>
+  </si>
+  <si>
+    <t>What's different</t>
+  </si>
+  <si>
+    <t>Launch (Product/Feature)</t>
+  </si>
+  <si>
+    <t>Full</t>
+  </si>
+  <si>
+    <t>The baseline - this is what the RACI's 8 stages are built around.</t>
+  </si>
+  <si>
+    <t>New Standalone Landing Page</t>
+  </si>
+  <si>
+    <t>Light</t>
+  </si>
+  <si>
+    <t>Skip</t>
+  </si>
+  <si>
+    <t>Skips Activation Planning entirely - this isn't a campaign, just a page.</t>
+  </si>
+  <si>
+    <t>Content-Only Piece</t>
+  </si>
+  <si>
+    <t>Lightest of all types - mostly just Content + SEO, skip most cross-team stages.</t>
+  </si>
+  <si>
+    <t>Existing Page Update</t>
+  </si>
+  <si>
+    <t>Smallest footprint - often just Web, no content pipeline unless copy changes.</t>
+  </si>
+  <si>
+    <t>Creative-Only Request</t>
+  </si>
+  <si>
+    <t>No campaign machinery - just Creative, with conditional Brand sign-off.</t>
+  </si>
+  <si>
+    <t>Campaign (non-launch)</t>
+  </si>
+  <si>
+    <t>Activation Planning and Post-Launch reporting are the heart of this one - Positioning is usually inherited, not created fresh.</t>
+  </si>
+  <si>
+    <t>Event / Webinar</t>
+  </si>
+  <si>
+    <t>Runs mostly independent of launch machinery unless explicitly tied to one.</t>
+  </si>
+  <si>
+    <t>PR / Thought Leadership</t>
+  </si>
+  <si>
+    <t>Positioning &amp; Narrative and Review &amp; Approval carry more weight here - Brand's involvement is central, not optional.</t>
+  </si>
+  <si>
+    <t>Community Platform Build</t>
+  </si>
+  <si>
+    <t>Mostly a Production-and-Launch exercise - no activation planning or centralized brief since it's usually one BU.</t>
+  </si>
+  <si>
+    <t>Partner Co-Marketing Asset</t>
+  </si>
+  <si>
+    <t>Activation Planning here is really the unresolved routing/attribution question, not classic channel planning.</t>
+  </si>
+  <si>
+    <t>SEO Technical Work</t>
+  </si>
+  <si>
+    <t>No content or creative involvement at all - purely SEO (+Web if it touches a live page).</t>
+  </si>
+  <si>
+    <t>Email / Lifecycle Campaign</t>
+  </si>
+  <si>
+    <t>Similar shape to Campaign but single-channel - no activation-planning decision since the channel is already fixed.</t>
+  </si>
+  <si>
+    <t>Legend:</t>
+  </si>
+  <si>
+    <t>full stage applies</t>
+  </si>
+  <si>
+    <t>lighter/partial involvement</t>
+  </si>
+  <si>
+    <t>does not apply for this project type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1918,6 +2024,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF082521"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF363432"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF898781"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -2002,7 +2137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2029,14 +2164,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2057,6 +2184,22 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4348,34 +4491,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21.3" x14ac:dyDescent="0.85">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="14" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="15" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="1.4">
-      <c r="A4" s="20">
+      <c r="A4" s="16">
         <v>17</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="18">
         <v>8</v>
       </c>
-      <c r="C4" s="24">
+      <c r="C4" s="20">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="21" t="s">
         <v>172</v>
       </c>
     </row>
@@ -4584,6 +4727,474 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77218B90-BED6-42B1-9427-0EA34C679710}">
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="26.578125" customWidth="1"/>
+    <col min="2" max="9" width="14.578125" customWidth="1"/>
+    <col min="10" max="10" width="55.578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="18.3" x14ac:dyDescent="0.7">
+      <c r="A1" s="27" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="J5" s="28" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="J7" s="28" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="J9" s="28" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="J10" s="28" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="J11" s="28" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="J12" s="28" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="J13" s="28" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="J15" s="28" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="J16" s="28" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="26" t="s">
+        <v>206</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="C18" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="30" t="s">
+        <v>183</v>
+      </c>
+      <c r="C19" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="31" t="s">
+        <v>184</v>
+      </c>
+      <c r="C20" t="s">
+        <v>209</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{066AAA2B-C07C-4CB2-AB30-85AA3DD73DAB}">
   <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -4636,18 +5247,18 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
@@ -4778,18 +5389,18 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
@@ -4920,18 +5531,18 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
@@ -5190,18 +5801,18 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="25"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="5" t="s">
@@ -5241,60 +5852,60 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
     </row>
     <row r="30" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
     </row>
     <row r="32" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="15"/>
-      <c r="J32" s="15"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5312,7 +5923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98F8F183-0888-4E35-ACCC-4B4021D90D9F}">
   <dimension ref="A1:H137"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>

<commit_message>
Improve Executive Summary tab: 4th KPI tile, conflict headlines, date stamp
- Added Project Type Guide KPI tile so the summary reflects the whole
  workbook, not just the launch process
- Open Conflicts now listed as full one-line headlines directly on the
  summary, not just a count requiring a tab switch
- Added a Last Updated date stamp
- Fixed a chart-anchoring bug where both charts were positioned on top
  of each other, and chart 2 was stretching when column widths changed
</commit_message>
<xml_diff>
--- a/marketing-ownership-map.xlsx
+++ b/marketing-ownership-map.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LRUSIN~1\AppData\Local\Temp\claude\c--Users-lrusinova-OneDrive---QuickBase-Documents-Project-Management-MCP\abf0f386-0ae7-411b-800d-e81e7586b212\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAA708C2-042D-4FF9-B4C2-97C5AB71F5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F973499D-1305-4FED-922A-1E69E2EB9B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{6BE01299-3AA2-44C9-B560-36F384A9188D}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{6BE01299-3AA2-44C9-B560-36F384A9188D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="3" r:id="rId1"/>
+    <sheet name="Executive Summary" sheetId="5" r:id="rId1"/>
     <sheet name="Project Type Guide" sheetId="4" r:id="rId2"/>
     <sheet name="Ownership Matrix" sheetId="1" r:id="rId3"/>
     <sheet name="Data" sheetId="2" r:id="rId4"/>
@@ -1264,7 +1264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1290" uniqueCount="217">
   <si>
     <t>Marketing Ownership Map - RACI Matrix (Working Draft)</t>
   </si>
@@ -1773,9 +1773,6 @@
     <t>Marketing Ownership Map - Executive Summary</t>
   </si>
   <si>
-    <t>For SLT review - see Ownership Matrix tab for full detail, Data tab for the filterable flat view</t>
-  </si>
-  <si>
     <t>Teams mapped across the launch process</t>
   </si>
   <si>
@@ -1894,13 +1891,37 @@
   </si>
   <si>
     <t>does not apply for this project type</t>
+  </si>
+  <si>
+    <t>For SLT review - see Project Type Guide for how this scales down for smaller work, Ownership Matrix for full detail, Data tab for the filterable flat view</t>
+  </si>
+  <si>
+    <t>Last updated: August 7, 2026</t>
+  </si>
+  <si>
+    <t>Project types mapped (see Project Type Guide)</t>
+  </si>
+  <si>
+    <t>1. Activation Planning: PMM vs. Demand Gen - both show R, no agreed Accountable.</t>
+  </si>
+  <si>
+    <t>2. Production: PMM vs. Brand/Positioning vs. Content - messaging/copy ownership unresolved. The single biggest open question on the board.</t>
+  </si>
+  <si>
+    <t>3. Paid Media vs. Demand Gen - unclear whether paid activation is a Demand Gen sub-decision or owned directly by Paid Media.</t>
+  </si>
+  <si>
+    <t>4. Partner Marketing - routing/attribution ownership open; Channel Leader role not yet filled.</t>
+  </si>
+  <si>
+    <t>Supporting detail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2053,6 +2074,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF898781"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -2137,7 +2166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2184,6 +2213,14 @@
     <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2192,14 +2229,14 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2323,7 +2360,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Executive Summary'!$G$8</c:f>
+              <c:f>'Executive Summary'!$G$15</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2344,7 +2381,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Summary'!$F$9:$F$25</c:f>
+              <c:f>'Executive Summary'!$F$16:$F$32</c:f>
               <c:strCache>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
@@ -2403,7 +2440,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Summary'!$G$9:$G$25</c:f>
+              <c:f>'Executive Summary'!$G$16:$G$32</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="17"/>
@@ -2463,7 +2500,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D468-41F5-BD81-2D150BADEADE}"/>
+              <c16:uniqueId val="{00000000-2C28-4F63-B6FE-34DC79C9D6EF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2476,11 +2513,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="182"/>
-        <c:axId val="1480255792"/>
-        <c:axId val="1480245712"/>
+        <c:axId val="1927333471"/>
+        <c:axId val="1927334911"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1480255792"/>
+        <c:axId val="1927333471"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2523,7 +2560,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480245712"/>
+        <c:crossAx val="1927334911"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2531,7 +2568,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1480245712"/>
+        <c:axId val="1927334911"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2582,7 +2619,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480255792"/>
+        <c:crossAx val="1927333471"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2719,7 +2756,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Executive Summary'!$J$8</c:f>
+              <c:f>'Executive Summary'!$J$15</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2740,7 +2777,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'Executive Summary'!$I$9:$I$16</c:f>
+              <c:f>'Executive Summary'!$I$16:$I$23</c:f>
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
@@ -2772,7 +2809,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Executive Summary'!$J$9:$J$16</c:f>
+              <c:f>'Executive Summary'!$J$16:$J$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -2805,7 +2842,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AC4F-4A36-97C7-8B31F1AA5EDE}"/>
+              <c16:uniqueId val="{00000000-C445-44B9-9506-258870A7B0D5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2819,11 +2856,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1480252912"/>
-        <c:axId val="1480247152"/>
+        <c:axId val="1927329631"/>
+        <c:axId val="1927327711"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1480252912"/>
+        <c:axId val="1927329631"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2866,7 +2903,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480247152"/>
+        <c:crossAx val="1927327711"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2874,7 +2911,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1480247152"/>
+        <c:axId val="1927327711"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2925,7 +2962,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480252912"/>
+        <c:crossAx val="1927329631"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4071,17 +4108,17 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1267460</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:colOff>1557020</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>111760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4089,7 +4126,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{628E7048-07B3-D9A3-AC58-6E93E3F8B46A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{845C40EB-1E42-C301-DC15-FD3BE36BB47D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4107,17 +4144,17 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>176530</xdr:colOff>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>372110</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1356360</xdr:colOff>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>111760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4125,7 +4162,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{398B62D7-F564-8594-BA55-71B7D9E88455}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{159423BA-7770-BD58-022E-CAF199A7DB9D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4479,11 +4516,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70A489AD-4DDD-4622-A71F-CC7D1D665555}">
-  <dimension ref="A1:J25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A4A1782-B0F0-4A80-B5B0-6DF2F503376B}">
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="3" width="24.578125" customWidth="1"/>
+    <col min="1" max="4" width="22.578125" customWidth="1"/>
     <col min="6" max="6" width="20.578125" customWidth="1"/>
     <col min="7" max="7" width="10.578125" customWidth="1"/>
     <col min="9" max="9" width="26.578125" customWidth="1"/>
@@ -4497,230 +4534,289 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="15" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="32" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="1.4">
+      <c r="A5" s="16">
+        <v>17</v>
+      </c>
+      <c r="B5" s="18">
+        <v>8</v>
+      </c>
+      <c r="C5" s="33">
+        <v>12</v>
+      </c>
+      <c r="D5" s="20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="34" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="17" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="1.4">
-      <c r="A4" s="16">
-        <v>17</v>
-      </c>
-      <c r="B4" s="18">
-        <v>8</v>
-      </c>
-      <c r="C4" s="20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="17" t="s">
+      <c r="B6" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="C6" s="34" t="s">
+        <v>211</v>
+      </c>
+      <c r="D6" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="C5" s="21" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F8" t="s">
-        <v>2</v>
-      </c>
-      <c r="G8" t="s">
-        <v>173</v>
-      </c>
-      <c r="I8" t="s">
-        <v>62</v>
-      </c>
-      <c r="J8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="I9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J9">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10">
-        <v>3</v>
-      </c>
-      <c r="I10" t="s">
-        <v>5</v>
-      </c>
-      <c r="J10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F11" t="s">
-        <v>43</v>
-      </c>
-      <c r="G11">
-        <v>3</v>
-      </c>
-      <c r="I11" t="s">
-        <v>6</v>
-      </c>
-      <c r="J11">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12">
-        <v>3</v>
-      </c>
-      <c r="I12" t="s">
-        <v>7</v>
-      </c>
-      <c r="J12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F13" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13">
-        <v>3</v>
-      </c>
-      <c r="I13" t="s">
-        <v>8</v>
-      </c>
-      <c r="J13">
-        <v>15</v>
-      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.6">
+      <c r="A8" s="12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="28" t="s">
+        <v>212</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+    </row>
+    <row r="10" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="28" t="s">
+        <v>213</v>
+      </c>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+    </row>
+    <row r="11" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="28" t="s">
+        <v>214</v>
+      </c>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+    </row>
+    <row r="12" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="28" t="s">
+        <v>215</v>
+      </c>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="F14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14">
-        <v>2</v>
-      </c>
-      <c r="I14" t="s">
-        <v>9</v>
-      </c>
-      <c r="J14">
-        <v>15</v>
+      <c r="A14" s="35" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F15" t="s">
-        <v>32</v>
-      </c>
-      <c r="G15">
         <v>2</v>
       </c>
+      <c r="G15" t="s">
+        <v>172</v>
+      </c>
       <c r="I15" t="s">
-        <v>10</v>
-      </c>
-      <c r="J15">
-        <v>13</v>
+        <v>62</v>
+      </c>
+      <c r="J15" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F16" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J16">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="6:7" x14ac:dyDescent="0.55000000000000004">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="6:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F17" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="G17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="6:7" x14ac:dyDescent="0.55000000000000004">
+        <v>3</v>
+      </c>
+      <c r="I17" t="s">
+        <v>5</v>
+      </c>
+      <c r="J17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="6:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F18" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="6:7" x14ac:dyDescent="0.55000000000000004">
+        <v>3</v>
+      </c>
+      <c r="I18" t="s">
+        <v>6</v>
+      </c>
+      <c r="J18">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="6:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="6:7" x14ac:dyDescent="0.55000000000000004">
+        <v>3</v>
+      </c>
+      <c r="I19" t="s">
+        <v>7</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="6:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="6:7" x14ac:dyDescent="0.55000000000000004">
+        <v>3</v>
+      </c>
+      <c r="I20" t="s">
+        <v>8</v>
+      </c>
+      <c r="J20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="6:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F21" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="6:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="I21" t="s">
+        <v>9</v>
+      </c>
+      <c r="J21">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="6:10" x14ac:dyDescent="0.55000000000000004">
       <c r="F22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="I22" t="s">
+        <v>10</v>
+      </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F23" t="s">
+        <v>35</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="I23" t="s">
+        <v>11</v>
+      </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F24" t="s">
+        <v>37</v>
+      </c>
+      <c r="G24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F25" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F26" t="s">
+        <v>41</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F27" t="s">
+        <v>49</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F28" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F29" t="s">
         <v>23</v>
       </c>
-      <c r="G22">
+      <c r="G29">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="6:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="F23" t="s">
+    <row r="30" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F30" t="s">
         <v>26</v>
       </c>
-      <c r="G23">
+      <c r="G30">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="6:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="F24" t="s">
+    <row r="31" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F31" t="s">
         <v>28</v>
       </c>
-      <c r="G24">
+      <c r="G31">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="6:7" x14ac:dyDescent="0.55000000000000004">
-      <c r="F25" t="s">
+    <row r="32" spans="6:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="F32" t="s">
         <v>30</v>
       </c>
-      <c r="G25">
+      <c r="G32">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -4737,18 +4833,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.3" x14ac:dyDescent="0.7">
-      <c r="A1" s="27" t="s">
-        <v>175</v>
+      <c r="A1" s="23" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>4</v>
@@ -4775,418 +4871,418 @@
         <v>11</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="J5" s="24" t="s">
         <v>180</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="J5" s="28" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="E6" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J6" s="24" t="s">
         <v>184</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="J6" s="28" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="J7" s="24" t="s">
         <v>186</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="J7" s="28" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="J8" s="24" t="s">
         <v>188</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="J8" s="28" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="J9" s="24" t="s">
         <v>190</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="J9" s="28" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="J10" s="24" t="s">
         <v>192</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="J10" s="28" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="J11" s="24" t="s">
         <v>194</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="J11" s="28" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J12" s="24" t="s">
         <v>196</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="J12" s="28" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J13" s="24" t="s">
         <v>198</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="J13" s="28" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="J14" s="24" t="s">
         <v>200</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="J14" s="28" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J15" s="24" t="s">
         <v>202</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="J15" s="28" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="J16" s="24" t="s">
         <v>204</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G16" s="8" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>179</v>
+      </c>
+      <c r="C18" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="C19" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="H16" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="J16" s="28" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="26" t="s">
-        <v>206</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>180</v>
-      </c>
-      <c r="C18" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="B19" s="30" t="s">
-        <v>183</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
         <v>208</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="B20" s="31" t="s">
-        <v>184</v>
-      </c>
-      <c r="C20" t="s">
-        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -5247,18 +5343,18 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
@@ -5389,18 +5485,18 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="25"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
@@ -5531,18 +5627,18 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
@@ -5801,18 +5897,18 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="5" t="s">
@@ -5852,60 +5948,60 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
     </row>
     <row r="30" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="29"/>
+      <c r="I30" s="29"/>
+      <c r="J30" s="29"/>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="23"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
     </row>
     <row r="32" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
Add Customer Story/Case Study and Sales Enablement Asset project types (14 total)
</commit_message>
<xml_diff>
--- a/marketing-ownership-map.xlsx
+++ b/marketing-ownership-map.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LRUSIN~1\AppData\Local\Temp\claude\c--Users-lrusinova-OneDrive---QuickBase-Documents-Project-Management-MCP\abf0f386-0ae7-411b-800d-e81e7586b212\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F973499D-1305-4FED-922A-1E69E2EB9B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674B75B3-42B8-4763-AFB8-98EE3F4FD91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{6BE01299-3AA2-44C9-B560-36F384A9188D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="5" r:id="rId1"/>
-    <sheet name="Project Type Guide" sheetId="4" r:id="rId2"/>
+    <sheet name="Executive Summary" sheetId="7" r:id="rId1"/>
+    <sheet name="Project Type Guide" sheetId="6" r:id="rId2"/>
     <sheet name="Ownership Matrix" sheetId="1" r:id="rId3"/>
     <sheet name="Data" sheetId="2" r:id="rId4"/>
   </sheets>
@@ -1264,7 +1264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1290" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="221">
   <si>
     <t>Marketing Ownership Map - RACI Matrix (Working Draft)</t>
   </si>
@@ -1915,6 +1915,18 @@
   </si>
   <si>
     <t>Supporting detail</t>
+  </si>
+  <si>
+    <t>Customer Story / Case Study</t>
+  </si>
+  <si>
+    <t>Unlike other content, needs the customer's own sign-off before it can publish - that approval loop is the real bottleneck, not internal review.</t>
+  </si>
+  <si>
+    <t>Sales Enablement Asset</t>
+  </si>
+  <si>
+    <t>Internal-facing, not customer-facing - no public launch execution; PMM usually owns it start to finish with light Content/Creative polish.</t>
   </si>
 </sst>
 </file>
@@ -2221,6 +2233,14 @@
     <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2229,14 +2249,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2500,7 +2512,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2C28-4F63-B6FE-34DC79C9D6EF}"/>
+              <c16:uniqueId val="{00000000-3138-4869-849D-DFD151A334E8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2513,11 +2525,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="182"/>
-        <c:axId val="1927333471"/>
-        <c:axId val="1927334911"/>
+        <c:axId val="238520911"/>
+        <c:axId val="238529551"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1927333471"/>
+        <c:axId val="238520911"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2560,7 +2572,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1927334911"/>
+        <c:crossAx val="238529551"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2568,7 +2580,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1927334911"/>
+        <c:axId val="238529551"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2619,7 +2631,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1927333471"/>
+        <c:crossAx val="238520911"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2842,7 +2854,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C445-44B9-9506-258870A7B0D5}"/>
+              <c16:uniqueId val="{00000000-EB42-41D5-B9A3-28F8F7FCC5DC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2856,11 +2868,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1927329631"/>
-        <c:axId val="1927327711"/>
+        <c:axId val="238530031"/>
+        <c:axId val="238518511"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1927329631"/>
+        <c:axId val="238530031"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2903,7 +2915,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1927327711"/>
+        <c:crossAx val="238518511"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2911,7 +2923,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1927327711"/>
+        <c:axId val="238518511"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2962,7 +2974,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1927329631"/>
+        <c:crossAx val="238530031"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4126,7 +4138,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{845C40EB-1E42-C301-DC15-FD3BE36BB47D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8478AF3D-B0EE-5D9F-96D8-E71C7A4B4CC9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4162,7 +4174,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{159423BA-7770-BD58-022E-CAF199A7DB9D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{818AF01E-6438-916D-1A02-191DF4C7D4E8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4516,7 +4528,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A4A1782-B0F0-4A80-B5B0-6DF2F503376B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC05E435-C543-472B-BA10-01E2880EEBEB}">
   <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -4538,7 +4550,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="28" t="s">
         <v>210</v>
       </c>
     </row>
@@ -4549,8 +4561,8 @@
       <c r="B5" s="18">
         <v>8</v>
       </c>
-      <c r="C5" s="33">
-        <v>12</v>
+      <c r="C5" s="29">
+        <v>14</v>
       </c>
       <c r="D5" s="20">
         <v>4</v>
@@ -4563,7 +4575,7 @@
       <c r="B6" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="30" t="s">
         <v>211</v>
       </c>
       <c r="D6" s="21" t="s">
@@ -4576,39 +4588,39 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
     </row>
     <row r="10" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
     </row>
     <row r="11" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="32" t="s">
         <v>214</v>
       </c>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
     </row>
     <row r="12" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="35" t="s">
+      <c r="A14" s="31" t="s">
         <v>216</v>
       </c>
     </row>
@@ -4823,8 +4835,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77218B90-BED6-42B1-9427-0EA34C679710}">
-  <dimension ref="A1:J20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099D435-D650-43CE-A7D2-53BDD00EBC1E}">
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="26.578125" customWidth="1"/>
@@ -5258,30 +5270,94 @@
         <v>204</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="22" t="s">
+    <row r="17" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J17" s="24" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="J18" s="24" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B20" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C20" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="B19" s="26" t="s">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21" s="26" t="s">
         <v>182</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C21" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="B20" s="27" t="s">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C22" t="s">
         <v>208</v>
       </c>
     </row>
@@ -5343,18 +5419,18 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="35"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
@@ -5485,18 +5561,18 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="35"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
@@ -5627,18 +5703,18 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="31"/>
-      <c r="J15" s="31"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="5" t="s">
@@ -5897,18 +5973,18 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="30" t="s">
+      <c r="A24" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="31"/>
-      <c r="J24" s="31"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="35"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="5" t="s">
@@ -5948,60 +6024,60 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="29"/>
-      <c r="I29" s="29"/>
-      <c r="J29" s="29"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
     </row>
     <row r="30" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="29"/>
-      <c r="H30" s="29"/>
-      <c r="I30" s="29"/>
-      <c r="J30" s="29"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
     </row>
     <row r="31" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="29"/>
-      <c r="H31" s="29"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="29"/>
+      <c r="B31" s="33"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
     </row>
     <row r="32" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="29"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="29"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="33"/>
+      <c r="J32" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>